<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@4ad7a9c0c9d1a6f9fa1c0c018571a2df232022cb 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-CodeSystems.xlsx
+++ b/ValueSet-CodeSystems.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="54">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-10T07:56:47+00:00</t>
+    <t>2025-03-12T11:31:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -144,7 +144,28 @@
     <t>ICPC</t>
   </si>
   <si>
-    <t>urn:oid:2.16.840.1.113883.2.4.4.31.1</t>
+    <t>http://www.whocc.no/atc</t>
+  </si>
+  <si>
+    <t>ATC</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/sid/ndc</t>
+  </si>
+  <si>
+    <t>NDC</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/sid/cvx</t>
+  </si>
+  <si>
+    <t>CVX</t>
+  </si>
+  <si>
+    <t>urn:oid:2.16.840.1.113883.2.4.4.10</t>
+  </si>
+  <si>
+    <t>PRK</t>
   </si>
   <si>
     <t/>
@@ -425,7 +446,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -509,23 +530,47 @@
         <v>43</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@12988fe66657909315f2a996c831986357f9e3f4 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-CodeSystems.xlsx
+++ b/ValueSet-CodeSystems.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-07T10:44:48+00:00</t>
+    <t>2025-04-07T14:17:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -109,6 +109,12 @@
   </si>
   <si>
     <t>urn:oid:2.16.840.1.113883.6.96</t>
+  </si>
+  <si>
+    <t>urn:oid:2.16.840.1.113883.2.4.3.120.5.1</t>
+  </si>
+  <si>
+    <t>DHD DT</t>
   </si>
   <si>
     <t>urn:oid:2.16.840.1.113883.2.4.3.120.5.2</t>
@@ -446,7 +452,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -514,15 +520,15 @@
         <v>40</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s" s="2">
         <v>41</v>
-      </c>
-      <c r="B9" t="s" s="2">
-        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -562,15 +568,23 @@
         <v>51</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>53</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>